<commit_message>
Week 2 Part A and B
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="261">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="282">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -433,6 +433,9 @@
     <t xml:space="preserve">Record actual effort and evidence, not only completed readings. Time is an input; mastery is determined by the gates.</t>
   </si>
   <si>
+    <t xml:space="preserve">Use one row per study or practice block. Enter actual duration in minutes. Rows with Study ID EXAMPLE-001 are excluded from dashboard study hours.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Use one row per study or practice block. Row 6 is an example and is excluded from dashboard study hours; overwrite or delete it when ready.</t>
   </si>
   <si>
@@ -454,31 +457,92 @@
     <t xml:space="preserve">Evidence Link</t>
   </si>
   <si>
+    <t xml:space="preserve">Duration (min)</t>
+  </si>
+  <si>
     <t xml:space="preserve">W01-1</t>
   </si>
   <si>
-    <t xml:space="preserve">CFTC — Futures Market Basics</t>
+    <t xml:space="preserve">CFTC — Futures Market Basics
+NFA</t>
   </si>
   <si>
     <t xml:space="preserve">Yes</t>
   </si>
   <si>
+    <t xml:space="preserve">See week 1 note</t>
+  </si>
+  <si>
     <t xml:space="preserve">W01-2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CME – intro to future</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W01-3</t>
   </si>
   <si>
     <t xml:space="preserve">Part C</t>
   </si>
   <si>
-    <t xml:space="preserve">W01-3</t>
+    <t xml:space="preserve">W01-4</t>
   </si>
   <si>
     <t xml:space="preserve">Part D</t>
   </si>
   <si>
-    <t xml:space="preserve">W01-4</t>
+    <t xml:space="preserve">W01-5</t>
   </si>
   <si>
     <t xml:space="preserve">Install Windows 11; Review notions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W01-6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W01-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Book 01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W01-8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quiz F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer initial questions from GPT about risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Answer question about risk</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Notional value, calculate tick value and total $</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See week 2 assignment.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P&amp;L from fills</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -815,22 +879,27 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="13">
+  <numFmts count="18">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="\$#,##0"/>
-    <numFmt numFmtId="166" formatCode="0.00%"/>
-    <numFmt numFmtId="167" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\);\-"/>
-    <numFmt numFmtId="168" formatCode="\$#,##0.00"/>
-    <numFmt numFmtId="169" formatCode="0.00;[RED]\(0.00\);\-"/>
-    <numFmt numFmtId="170" formatCode="0.0"/>
-    <numFmt numFmtId="171" formatCode="0.0%"/>
-    <numFmt numFmtId="172" formatCode="0"/>
-    <numFmt numFmtId="173" formatCode="yyyy/mm/dd"/>
-    <numFmt numFmtId="174" formatCode="hh:mm"/>
-    <numFmt numFmtId="175" formatCode="0.00####"/>
-    <numFmt numFmtId="176" formatCode="0%"/>
+    <numFmt numFmtId="165" formatCode="_ * #,##0.00_)\ _$_ ;_ * \(#,##0.00&quot;) &quot;_$_ ;_ * \-??_)\ _$_ ;_ @_ "/>
+    <numFmt numFmtId="166" formatCode="_ * #,##0_)\ _$_ ;_ * \(#,##0&quot;) &quot;_$_ ;_ * \-_)\ _$_ ;_ @_ "/>
+    <numFmt numFmtId="167" formatCode="_ * #,##0.00_)&quot; $&quot;_ ;_ * \(#,##0.00&quot;) $&quot;_ ;_ * \-??_)&quot; $&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="168" formatCode="_ * #,##0_)&quot; $&quot;_ ;_ * \(#,##0&quot;) $&quot;_ ;_ * \-_)&quot; $&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="169" formatCode="0\ %"/>
+    <numFmt numFmtId="170" formatCode="\$#,##0"/>
+    <numFmt numFmtId="171" formatCode="0.00%"/>
+    <numFmt numFmtId="172" formatCode="\$#,##0.00;[RED]&quot;($&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="173" formatCode="\$#,##0.00"/>
+    <numFmt numFmtId="174" formatCode="0.00;[RED]\(0.00\);\-"/>
+    <numFmt numFmtId="175" formatCode="0.0"/>
+    <numFmt numFmtId="176" formatCode="0.0%"/>
+    <numFmt numFmtId="177" formatCode="0"/>
+    <numFmt numFmtId="178" formatCode="yyyy/mm/dd"/>
+    <numFmt numFmtId="179" formatCode="hh:mm"/>
+    <numFmt numFmtId="180" formatCode="0.00####"/>
+    <numFmt numFmtId="181" formatCode="0%"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -851,6 +920,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
@@ -958,8 +1033,23 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <i val="true"/>
       <sz val="9"/>
+      <color rgb="FF182230"/>
+      <name val="Calibri"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FF182230"/>
       <name val="Calibri"/>
       <family val="0"/>
@@ -990,7 +1080,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1033,8 +1123,14 @@
         <bgColor rgb="FFE6E9EC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor rgb="FFF2F4F5"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="14">
+  <borders count="18">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1181,8 +1277,64 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFFFFFFF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFFFFFFF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFFFFFFF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFFFFFFF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD9E1E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1E8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E1E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD9E1E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E1E8"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9E1E8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FFD9E1E8"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E1E8"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E1E8"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="21">
+  <cellStyleXfs count="27">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1206,321 +1358,366 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="80">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="24" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="2" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="5" borderId="3" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="3" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="4" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="5" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="11" fillId="6" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="11" fillId="6" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="11" fillId="6" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="10" fillId="5" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="6" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="175" fontId="11" fillId="6" borderId="5" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="6" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="10" fillId="5" borderId="7" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="7" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="6" borderId="7" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="8" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="4" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="6" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="9" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="9" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="7" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="7" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="5" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="5" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="10" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="4" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="179" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="18" fillId="6" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="18" fillId="6" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="18" fillId="6" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="179" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="18" fillId="6" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="18" fillId="6" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="18" fillId="6" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="179" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="181" fontId="17" fillId="0" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="181" fontId="17" fillId="0" borderId="12" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="181" fontId="17" fillId="0" borderId="13" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="19" fillId="2" borderId="14" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="178" fontId="20" fillId="5" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="20" fillId="5" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="5" borderId="11" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="21" fillId="8" borderId="15" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="21" fillId="8" borderId="16" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="177" fontId="21" fillId="8" borderId="17" xfId="24" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="180" fontId="14" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="3" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="5" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="6" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="6" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="8" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="6" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="9" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="7" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="2" borderId="4" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="17" fillId="6" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="6" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="6" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="17" fillId="6" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="17" fillId="6" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="17" fillId="6" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="174" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="0" borderId="12" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="176" fontId="16" fillId="0" borderId="13" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="18" fillId="5" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="18" fillId="5" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="18" fillId="5" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="175" fontId="13" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="23" fillId="6" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="15" fillId="5" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="7" borderId="0" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="24" fillId="7" borderId="0" xfId="25" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
-  <cellStyles count="7">
+  <cellStyles count="13">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Comma" xfId="15" builtinId="3"/>
     <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Normal" xfId="20"/>
+    <cellStyle name="Comma" xfId="20"/>
+    <cellStyle name="Comma [0]" xfId="21"/>
+    <cellStyle name="Currency" xfId="22"/>
+    <cellStyle name="Currency [0]" xfId="23"/>
+    <cellStyle name="Normal" xfId="24"/>
+    <cellStyle name="Normal 1" xfId="25"/>
+    <cellStyle name="Percent" xfId="26"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
@@ -1690,7 +1887,7 @@
       <rgbColor rgb="FF8A5700"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF1F7A8C"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFD9E1E8"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
@@ -2249,9 +2446,9 @@
       <c r="G10" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H10" s="16" t="e">
-        <f aca="false">SUMIFS(#ref!,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>#NAME?</v>
+      <c r="H10" s="16" t="n">
+        <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
+        <v>10.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32473,7 +32670,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H205"/>
+  <dimension ref="A1:I205"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -32483,6 +32680,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="1" width="42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="62" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
@@ -32511,6 +32709,7 @@
       <c r="H1" s="2" t="s">
         <v>133</v>
       </c>
+      <c r="I1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
@@ -32537,36 +32736,38 @@
       <c r="H2" s="3" t="s">
         <v>134</v>
       </c>
+      <c r="I2" s="3"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="62" t="s">
+      <c r="A4" s="63" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="C4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="D4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="E4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="F4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="G4" s="62" t="s">
-        <v>135</v>
-      </c>
-      <c r="H4" s="62" t="s">
-        <v>135</v>
-      </c>
+      <c r="B4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="D4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="E4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="F4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="G4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="H4" s="63" t="s">
+        <v>136</v>
+      </c>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B5" s="33" t="s">
         <v>75</v>
@@ -32575,44 +32776,50 @@
         <v>77</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>141</v>
+        <v>142</v>
+      </c>
+      <c r="I5" s="64" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="44" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="63" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" s="64" t="n">
+      <c r="A6" s="65" t="s">
+        <v>144</v>
+      </c>
+      <c r="B6" s="66" t="n">
         <v>46258</v>
       </c>
-      <c r="C6" s="65" t="n">
+      <c r="C6" s="67" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="66" t="s">
-        <v>143</v>
-      </c>
-      <c r="E6" s="67" t="s">
-        <v>144</v>
-      </c>
-      <c r="F6" s="67"/>
-      <c r="G6" s="67"/>
-      <c r="H6" s="67"/>
+      <c r="D6" s="68" t="s">
+        <v>145</v>
+      </c>
+      <c r="E6" s="69" t="s">
+        <v>146</v>
+      </c>
+      <c r="F6" s="69"/>
+      <c r="G6" s="69"/>
+      <c r="H6" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="I6" s="70"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="44" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B7" s="45" t="n">
         <v>46265</v>
@@ -32620,17 +32827,24 @@
       <c r="C7" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="44" t="s">
-        <v>146</v>
-      </c>
-      <c r="E7" s="44"/>
+      <c r="D7" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F7" s="44"/>
       <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
+      <c r="H7" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="I7" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="44" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B8" s="45" t="n">
         <v>46265</v>
@@ -32639,16 +32853,23 @@
         <v>1</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>148</v>
-      </c>
-      <c r="E8" s="44"/>
+        <v>152</v>
+      </c>
+      <c r="E8" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F8" s="44"/>
       <c r="G8" s="44"/>
-      <c r="H8" s="44"/>
+      <c r="H8" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="I8" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="44" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B9" s="45" t="n">
         <v>46266</v>
@@ -32657,92 +32878,197 @@
         <v>1</v>
       </c>
       <c r="D9" s="44" t="s">
+        <v>154</v>
+      </c>
+      <c r="E9" s="44" t="s">
         <v>150</v>
       </c>
-      <c r="E9" s="44"/>
       <c r="F9" s="44"/>
       <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
+      <c r="H9" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="I9" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="44"/>
-      <c r="B10" s="45"/>
-      <c r="C10" s="48"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
+      <c r="A10" s="44" t="s">
+        <v>155</v>
+      </c>
+      <c r="B10" s="45" t="n">
+        <v>46267</v>
+      </c>
+      <c r="C10" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="44" t="s">
+        <v>156</v>
+      </c>
+      <c r="E10" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F10" s="44"/>
       <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="44"/>
-      <c r="B11" s="45"/>
-      <c r="C11" s="48"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
+      <c r="A11" s="44" t="s">
+        <v>157</v>
+      </c>
+      <c r="B11" s="45" t="n">
+        <v>46268</v>
+      </c>
+      <c r="C11" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="44" t="s">
+        <v>158</v>
+      </c>
+      <c r="E11" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F11" s="44"/>
       <c r="G11" s="44"/>
-      <c r="H11" s="44"/>
+      <c r="H11" s="44" t="s">
+        <v>159</v>
+      </c>
+      <c r="I11" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="44"/>
-      <c r="B12" s="45"/>
-      <c r="C12" s="48"/>
-      <c r="D12" s="44"/>
-      <c r="E12" s="44"/>
+      <c r="A12" s="44" t="s">
+        <v>160</v>
+      </c>
+      <c r="B12" s="45" t="n">
+        <v>46267</v>
+      </c>
+      <c r="C12" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="44" t="s">
+        <v>161</v>
+      </c>
+      <c r="E12" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F12" s="44"/>
       <c r="G12" s="44"/>
       <c r="H12" s="44"/>
+      <c r="I12" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="44"/>
-      <c r="B13" s="45"/>
-      <c r="C13" s="48"/>
-      <c r="D13" s="44"/>
-      <c r="E13" s="44"/>
+      <c r="A13" s="44" t="s">
+        <v>162</v>
+      </c>
+      <c r="B13" s="45" t="n">
+        <v>46272</v>
+      </c>
+      <c r="C13" s="48" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="44" t="s">
+        <v>163</v>
+      </c>
+      <c r="E13" s="44" t="s">
+        <v>150</v>
+      </c>
       <c r="F13" s="44"/>
       <c r="G13" s="44"/>
-      <c r="H13" s="44"/>
+      <c r="H13" s="44" t="s">
+        <v>147</v>
+      </c>
+      <c r="I13" s="71" t="n">
+        <v>120</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="44"/>
       <c r="B14" s="45"/>
-      <c r="C14" s="48"/>
-      <c r="D14" s="44"/>
-      <c r="E14" s="44"/>
+      <c r="C14" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="44" t="s">
+        <v>164</v>
+      </c>
+      <c r="E14" s="44" t="s">
+        <v>165</v>
+      </c>
       <c r="F14" s="44"/>
       <c r="G14" s="44"/>
       <c r="H14" s="44"/>
+      <c r="I14" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="44"/>
       <c r="B15" s="45"/>
-      <c r="C15" s="48"/>
-      <c r="D15" s="44"/>
-      <c r="E15" s="44"/>
+      <c r="C15" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="44" t="s">
+        <v>166</v>
+      </c>
+      <c r="E15" s="44" t="s">
+        <v>146</v>
+      </c>
       <c r="F15" s="44"/>
       <c r="G15" s="44"/>
       <c r="H15" s="44"/>
+      <c r="I15" s="71"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="44"/>
       <c r="B16" s="45"/>
-      <c r="C16" s="48"/>
-      <c r="D16" s="44"/>
-      <c r="E16" s="44"/>
-      <c r="F16" s="44"/>
+      <c r="C16" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" s="44" t="s">
+        <v>167</v>
+      </c>
+      <c r="E16" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F16" s="44" t="s">
+        <v>168</v>
+      </c>
       <c r="G16" s="44"/>
-      <c r="H16" s="44"/>
+      <c r="H16" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="I16" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="44"/>
       <c r="B17" s="45"/>
-      <c r="C17" s="48"/>
-      <c r="D17" s="44"/>
-      <c r="E17" s="44"/>
-      <c r="F17" s="44"/>
+      <c r="C17" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D17" s="44" t="s">
+        <v>170</v>
+      </c>
+      <c r="E17" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F17" s="44" t="s">
+        <v>171</v>
+      </c>
       <c r="G17" s="44"/>
-      <c r="H17" s="44"/>
+      <c r="H17" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="I17" s="71" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="44"/>
@@ -32753,6 +33079,7 @@
       <c r="F18" s="44"/>
       <c r="G18" s="44"/>
       <c r="H18" s="44"/>
+      <c r="I18" s="71"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="44"/>
@@ -32763,6 +33090,7 @@
       <c r="F19" s="44"/>
       <c r="G19" s="44"/>
       <c r="H19" s="44"/>
+      <c r="I19" s="71"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="44"/>
@@ -32773,6 +33101,7 @@
       <c r="F20" s="44"/>
       <c r="G20" s="44"/>
       <c r="H20" s="44"/>
+      <c r="I20" s="71"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="44"/>
@@ -32783,6 +33112,7 @@
       <c r="F21" s="44"/>
       <c r="G21" s="44"/>
       <c r="H21" s="44"/>
+      <c r="I21" s="71"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="44"/>
@@ -32793,6 +33123,7 @@
       <c r="F22" s="44"/>
       <c r="G22" s="44"/>
       <c r="H22" s="44"/>
+      <c r="I22" s="71"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="44"/>
@@ -32803,6 +33134,7 @@
       <c r="F23" s="44"/>
       <c r="G23" s="44"/>
       <c r="H23" s="44"/>
+      <c r="I23" s="71"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="44"/>
@@ -32813,6 +33145,7 @@
       <c r="F24" s="44"/>
       <c r="G24" s="44"/>
       <c r="H24" s="44"/>
+      <c r="I24" s="71"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="44"/>
@@ -32823,6 +33156,7 @@
       <c r="F25" s="44"/>
       <c r="G25" s="44"/>
       <c r="H25" s="44"/>
+      <c r="I25" s="71"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="44"/>
@@ -32833,6 +33167,7 @@
       <c r="F26" s="44"/>
       <c r="G26" s="44"/>
       <c r="H26" s="44"/>
+      <c r="I26" s="71"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="44"/>
@@ -32843,6 +33178,7 @@
       <c r="F27" s="44"/>
       <c r="G27" s="44"/>
       <c r="H27" s="44"/>
+      <c r="I27" s="71"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="44"/>
@@ -32853,6 +33189,7 @@
       <c r="F28" s="44"/>
       <c r="G28" s="44"/>
       <c r="H28" s="44"/>
+      <c r="I28" s="71"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="44"/>
@@ -32863,6 +33200,7 @@
       <c r="F29" s="44"/>
       <c r="G29" s="44"/>
       <c r="H29" s="44"/>
+      <c r="I29" s="71"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="44"/>
@@ -32873,6 +33211,7 @@
       <c r="F30" s="44"/>
       <c r="G30" s="44"/>
       <c r="H30" s="44"/>
+      <c r="I30" s="71"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="44"/>
@@ -32883,6 +33222,7 @@
       <c r="F31" s="44"/>
       <c r="G31" s="44"/>
       <c r="H31" s="44"/>
+      <c r="I31" s="71"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="44"/>
@@ -32893,6 +33233,7 @@
       <c r="F32" s="44"/>
       <c r="G32" s="44"/>
       <c r="H32" s="44"/>
+      <c r="I32" s="71"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="44"/>
@@ -32903,6 +33244,7 @@
       <c r="F33" s="44"/>
       <c r="G33" s="44"/>
       <c r="H33" s="44"/>
+      <c r="I33" s="71"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="44"/>
@@ -32913,6 +33255,7 @@
       <c r="F34" s="44"/>
       <c r="G34" s="44"/>
       <c r="H34" s="44"/>
+      <c r="I34" s="71"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="44"/>
@@ -32923,6 +33266,7 @@
       <c r="F35" s="44"/>
       <c r="G35" s="44"/>
       <c r="H35" s="44"/>
+      <c r="I35" s="71"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="44"/>
@@ -32933,6 +33277,7 @@
       <c r="F36" s="44"/>
       <c r="G36" s="44"/>
       <c r="H36" s="44"/>
+      <c r="I36" s="71"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="44"/>
@@ -32943,6 +33288,7 @@
       <c r="F37" s="44"/>
       <c r="G37" s="44"/>
       <c r="H37" s="44"/>
+      <c r="I37" s="71"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="44"/>
@@ -32953,6 +33299,7 @@
       <c r="F38" s="44"/>
       <c r="G38" s="44"/>
       <c r="H38" s="44"/>
+      <c r="I38" s="71"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="44"/>
@@ -32963,6 +33310,7 @@
       <c r="F39" s="44"/>
       <c r="G39" s="44"/>
       <c r="H39" s="44"/>
+      <c r="I39" s="71"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="44"/>
@@ -32973,6 +33321,7 @@
       <c r="F40" s="44"/>
       <c r="G40" s="44"/>
       <c r="H40" s="44"/>
+      <c r="I40" s="71"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="44"/>
@@ -32983,6 +33332,7 @@
       <c r="F41" s="44"/>
       <c r="G41" s="44"/>
       <c r="H41" s="44"/>
+      <c r="I41" s="71"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="44"/>
@@ -32993,6 +33343,7 @@
       <c r="F42" s="44"/>
       <c r="G42" s="44"/>
       <c r="H42" s="44"/>
+      <c r="I42" s="71"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="44"/>
@@ -33003,6 +33354,7 @@
       <c r="F43" s="44"/>
       <c r="G43" s="44"/>
       <c r="H43" s="44"/>
+      <c r="I43" s="71"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="44"/>
@@ -33013,6 +33365,7 @@
       <c r="F44" s="44"/>
       <c r="G44" s="44"/>
       <c r="H44" s="44"/>
+      <c r="I44" s="71"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="44"/>
@@ -33023,6 +33376,7 @@
       <c r="F45" s="44"/>
       <c r="G45" s="44"/>
       <c r="H45" s="44"/>
+      <c r="I45" s="71"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="44"/>
@@ -33033,6 +33387,7 @@
       <c r="F46" s="44"/>
       <c r="G46" s="44"/>
       <c r="H46" s="44"/>
+      <c r="I46" s="71"/>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="44"/>
@@ -33043,6 +33398,7 @@
       <c r="F47" s="44"/>
       <c r="G47" s="44"/>
       <c r="H47" s="44"/>
+      <c r="I47" s="71"/>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="44"/>
@@ -33053,6 +33409,7 @@
       <c r="F48" s="44"/>
       <c r="G48" s="44"/>
       <c r="H48" s="44"/>
+      <c r="I48" s="71"/>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="44"/>
@@ -33063,6 +33420,7 @@
       <c r="F49" s="44"/>
       <c r="G49" s="44"/>
       <c r="H49" s="44"/>
+      <c r="I49" s="71"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="44"/>
@@ -33073,6 +33431,7 @@
       <c r="F50" s="44"/>
       <c r="G50" s="44"/>
       <c r="H50" s="44"/>
+      <c r="I50" s="71"/>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="44"/>
@@ -33083,6 +33442,7 @@
       <c r="F51" s="44"/>
       <c r="G51" s="44"/>
       <c r="H51" s="44"/>
+      <c r="I51" s="71"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="44"/>
@@ -33093,6 +33453,7 @@
       <c r="F52" s="44"/>
       <c r="G52" s="44"/>
       <c r="H52" s="44"/>
+      <c r="I52" s="71"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="44"/>
@@ -33103,6 +33464,7 @@
       <c r="F53" s="44"/>
       <c r="G53" s="44"/>
       <c r="H53" s="44"/>
+      <c r="I53" s="71"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="44"/>
@@ -33113,6 +33475,7 @@
       <c r="F54" s="44"/>
       <c r="G54" s="44"/>
       <c r="H54" s="44"/>
+      <c r="I54" s="71"/>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="44"/>
@@ -33123,6 +33486,7 @@
       <c r="F55" s="44"/>
       <c r="G55" s="44"/>
       <c r="H55" s="44"/>
+      <c r="I55" s="71"/>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="44"/>
@@ -33133,6 +33497,7 @@
       <c r="F56" s="44"/>
       <c r="G56" s="44"/>
       <c r="H56" s="44"/>
+      <c r="I56" s="71"/>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="44"/>
@@ -33143,6 +33508,7 @@
       <c r="F57" s="44"/>
       <c r="G57" s="44"/>
       <c r="H57" s="44"/>
+      <c r="I57" s="71"/>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="44"/>
@@ -33153,6 +33519,7 @@
       <c r="F58" s="44"/>
       <c r="G58" s="44"/>
       <c r="H58" s="44"/>
+      <c r="I58" s="71"/>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="44"/>
@@ -33163,6 +33530,7 @@
       <c r="F59" s="44"/>
       <c r="G59" s="44"/>
       <c r="H59" s="44"/>
+      <c r="I59" s="71"/>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="44"/>
@@ -33173,6 +33541,7 @@
       <c r="F60" s="44"/>
       <c r="G60" s="44"/>
       <c r="H60" s="44"/>
+      <c r="I60" s="71"/>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="44"/>
@@ -33183,6 +33552,7 @@
       <c r="F61" s="44"/>
       <c r="G61" s="44"/>
       <c r="H61" s="44"/>
+      <c r="I61" s="71"/>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="44"/>
@@ -33193,6 +33563,7 @@
       <c r="F62" s="44"/>
       <c r="G62" s="44"/>
       <c r="H62" s="44"/>
+      <c r="I62" s="71"/>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="44"/>
@@ -33203,6 +33574,7 @@
       <c r="F63" s="44"/>
       <c r="G63" s="44"/>
       <c r="H63" s="44"/>
+      <c r="I63" s="71"/>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="44"/>
@@ -33213,6 +33585,7 @@
       <c r="F64" s="44"/>
       <c r="G64" s="44"/>
       <c r="H64" s="44"/>
+      <c r="I64" s="71"/>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="44"/>
@@ -33223,6 +33596,7 @@
       <c r="F65" s="44"/>
       <c r="G65" s="44"/>
       <c r="H65" s="44"/>
+      <c r="I65" s="71"/>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="44"/>
@@ -33233,6 +33607,7 @@
       <c r="F66" s="44"/>
       <c r="G66" s="44"/>
       <c r="H66" s="44"/>
+      <c r="I66" s="71"/>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="44"/>
@@ -33243,6 +33618,7 @@
       <c r="F67" s="44"/>
       <c r="G67" s="44"/>
       <c r="H67" s="44"/>
+      <c r="I67" s="71"/>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="44"/>
@@ -33253,6 +33629,7 @@
       <c r="F68" s="44"/>
       <c r="G68" s="44"/>
       <c r="H68" s="44"/>
+      <c r="I68" s="71"/>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="44"/>
@@ -33263,6 +33640,7 @@
       <c r="F69" s="44"/>
       <c r="G69" s="44"/>
       <c r="H69" s="44"/>
+      <c r="I69" s="71"/>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="44"/>
@@ -33273,6 +33651,7 @@
       <c r="F70" s="44"/>
       <c r="G70" s="44"/>
       <c r="H70" s="44"/>
+      <c r="I70" s="71"/>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="44"/>
@@ -33283,6 +33662,7 @@
       <c r="F71" s="44"/>
       <c r="G71" s="44"/>
       <c r="H71" s="44"/>
+      <c r="I71" s="71"/>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="44"/>
@@ -33293,6 +33673,7 @@
       <c r="F72" s="44"/>
       <c r="G72" s="44"/>
       <c r="H72" s="44"/>
+      <c r="I72" s="71"/>
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="44"/>
@@ -33303,6 +33684,7 @@
       <c r="F73" s="44"/>
       <c r="G73" s="44"/>
       <c r="H73" s="44"/>
+      <c r="I73" s="71"/>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="44"/>
@@ -33313,6 +33695,7 @@
       <c r="F74" s="44"/>
       <c r="G74" s="44"/>
       <c r="H74" s="44"/>
+      <c r="I74" s="71"/>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="44"/>
@@ -33323,6 +33706,7 @@
       <c r="F75" s="44"/>
       <c r="G75" s="44"/>
       <c r="H75" s="44"/>
+      <c r="I75" s="71"/>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="44"/>
@@ -33333,6 +33717,7 @@
       <c r="F76" s="44"/>
       <c r="G76" s="44"/>
       <c r="H76" s="44"/>
+      <c r="I76" s="71"/>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="44"/>
@@ -33343,6 +33728,7 @@
       <c r="F77" s="44"/>
       <c r="G77" s="44"/>
       <c r="H77" s="44"/>
+      <c r="I77" s="71"/>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="44"/>
@@ -33353,6 +33739,7 @@
       <c r="F78" s="44"/>
       <c r="G78" s="44"/>
       <c r="H78" s="44"/>
+      <c r="I78" s="71"/>
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="44"/>
@@ -33363,6 +33750,7 @@
       <c r="F79" s="44"/>
       <c r="G79" s="44"/>
       <c r="H79" s="44"/>
+      <c r="I79" s="71"/>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="44"/>
@@ -33373,6 +33761,7 @@
       <c r="F80" s="44"/>
       <c r="G80" s="44"/>
       <c r="H80" s="44"/>
+      <c r="I80" s="71"/>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="44"/>
@@ -33383,6 +33772,7 @@
       <c r="F81" s="44"/>
       <c r="G81" s="44"/>
       <c r="H81" s="44"/>
+      <c r="I81" s="71"/>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="44"/>
@@ -33393,6 +33783,7 @@
       <c r="F82" s="44"/>
       <c r="G82" s="44"/>
       <c r="H82" s="44"/>
+      <c r="I82" s="71"/>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="44"/>
@@ -33403,6 +33794,7 @@
       <c r="F83" s="44"/>
       <c r="G83" s="44"/>
       <c r="H83" s="44"/>
+      <c r="I83" s="71"/>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="44"/>
@@ -33413,6 +33805,7 @@
       <c r="F84" s="44"/>
       <c r="G84" s="44"/>
       <c r="H84" s="44"/>
+      <c r="I84" s="71"/>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="44"/>
@@ -33423,6 +33816,7 @@
       <c r="F85" s="44"/>
       <c r="G85" s="44"/>
       <c r="H85" s="44"/>
+      <c r="I85" s="71"/>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="44"/>
@@ -33433,6 +33827,7 @@
       <c r="F86" s="44"/>
       <c r="G86" s="44"/>
       <c r="H86" s="44"/>
+      <c r="I86" s="71"/>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="44"/>
@@ -33443,6 +33838,7 @@
       <c r="F87" s="44"/>
       <c r="G87" s="44"/>
       <c r="H87" s="44"/>
+      <c r="I87" s="71"/>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="44"/>
@@ -33453,6 +33849,7 @@
       <c r="F88" s="44"/>
       <c r="G88" s="44"/>
       <c r="H88" s="44"/>
+      <c r="I88" s="71"/>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="44"/>
@@ -33463,6 +33860,7 @@
       <c r="F89" s="44"/>
       <c r="G89" s="44"/>
       <c r="H89" s="44"/>
+      <c r="I89" s="71"/>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="44"/>
@@ -33473,6 +33871,7 @@
       <c r="F90" s="44"/>
       <c r="G90" s="44"/>
       <c r="H90" s="44"/>
+      <c r="I90" s="71"/>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="44"/>
@@ -33483,6 +33882,7 @@
       <c r="F91" s="44"/>
       <c r="G91" s="44"/>
       <c r="H91" s="44"/>
+      <c r="I91" s="71"/>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="44"/>
@@ -33493,6 +33893,7 @@
       <c r="F92" s="44"/>
       <c r="G92" s="44"/>
       <c r="H92" s="44"/>
+      <c r="I92" s="71"/>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="44"/>
@@ -33503,6 +33904,7 @@
       <c r="F93" s="44"/>
       <c r="G93" s="44"/>
       <c r="H93" s="44"/>
+      <c r="I93" s="71"/>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="44"/>
@@ -33513,6 +33915,7 @@
       <c r="F94" s="44"/>
       <c r="G94" s="44"/>
       <c r="H94" s="44"/>
+      <c r="I94" s="71"/>
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="44"/>
@@ -33523,6 +33926,7 @@
       <c r="F95" s="44"/>
       <c r="G95" s="44"/>
       <c r="H95" s="44"/>
+      <c r="I95" s="71"/>
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="44"/>
@@ -33533,6 +33937,7 @@
       <c r="F96" s="44"/>
       <c r="G96" s="44"/>
       <c r="H96" s="44"/>
+      <c r="I96" s="71"/>
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="44"/>
@@ -33543,6 +33948,7 @@
       <c r="F97" s="44"/>
       <c r="G97" s="44"/>
       <c r="H97" s="44"/>
+      <c r="I97" s="71"/>
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="44"/>
@@ -33553,6 +33959,7 @@
       <c r="F98" s="44"/>
       <c r="G98" s="44"/>
       <c r="H98" s="44"/>
+      <c r="I98" s="71"/>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="44"/>
@@ -33563,6 +33970,7 @@
       <c r="F99" s="44"/>
       <c r="G99" s="44"/>
       <c r="H99" s="44"/>
+      <c r="I99" s="71"/>
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="44"/>
@@ -33573,6 +33981,7 @@
       <c r="F100" s="44"/>
       <c r="G100" s="44"/>
       <c r="H100" s="44"/>
+      <c r="I100" s="71"/>
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="44"/>
@@ -33583,6 +33992,7 @@
       <c r="F101" s="44"/>
       <c r="G101" s="44"/>
       <c r="H101" s="44"/>
+      <c r="I101" s="71"/>
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="44"/>
@@ -33593,6 +34003,7 @@
       <c r="F102" s="44"/>
       <c r="G102" s="44"/>
       <c r="H102" s="44"/>
+      <c r="I102" s="71"/>
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="44"/>
@@ -33603,6 +34014,7 @@
       <c r="F103" s="44"/>
       <c r="G103" s="44"/>
       <c r="H103" s="44"/>
+      <c r="I103" s="71"/>
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="44"/>
@@ -33613,6 +34025,7 @@
       <c r="F104" s="44"/>
       <c r="G104" s="44"/>
       <c r="H104" s="44"/>
+      <c r="I104" s="71"/>
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="44"/>
@@ -33623,6 +34036,7 @@
       <c r="F105" s="44"/>
       <c r="G105" s="44"/>
       <c r="H105" s="44"/>
+      <c r="I105" s="71"/>
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="44"/>
@@ -33633,6 +34047,7 @@
       <c r="F106" s="44"/>
       <c r="G106" s="44"/>
       <c r="H106" s="44"/>
+      <c r="I106" s="71"/>
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="44"/>
@@ -33643,6 +34058,7 @@
       <c r="F107" s="44"/>
       <c r="G107" s="44"/>
       <c r="H107" s="44"/>
+      <c r="I107" s="71"/>
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="44"/>
@@ -33653,6 +34069,7 @@
       <c r="F108" s="44"/>
       <c r="G108" s="44"/>
       <c r="H108" s="44"/>
+      <c r="I108" s="71"/>
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="44"/>
@@ -33663,6 +34080,7 @@
       <c r="F109" s="44"/>
       <c r="G109" s="44"/>
       <c r="H109" s="44"/>
+      <c r="I109" s="71"/>
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="44"/>
@@ -33673,6 +34091,7 @@
       <c r="F110" s="44"/>
       <c r="G110" s="44"/>
       <c r="H110" s="44"/>
+      <c r="I110" s="71"/>
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="44"/>
@@ -33683,6 +34102,7 @@
       <c r="F111" s="44"/>
       <c r="G111" s="44"/>
       <c r="H111" s="44"/>
+      <c r="I111" s="71"/>
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="44"/>
@@ -33693,6 +34113,7 @@
       <c r="F112" s="44"/>
       <c r="G112" s="44"/>
       <c r="H112" s="44"/>
+      <c r="I112" s="71"/>
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="44"/>
@@ -33703,6 +34124,7 @@
       <c r="F113" s="44"/>
       <c r="G113" s="44"/>
       <c r="H113" s="44"/>
+      <c r="I113" s="71"/>
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="44"/>
@@ -33713,6 +34135,7 @@
       <c r="F114" s="44"/>
       <c r="G114" s="44"/>
       <c r="H114" s="44"/>
+      <c r="I114" s="71"/>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="44"/>
@@ -33723,6 +34146,7 @@
       <c r="F115" s="44"/>
       <c r="G115" s="44"/>
       <c r="H115" s="44"/>
+      <c r="I115" s="71"/>
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="44"/>
@@ -33733,6 +34157,7 @@
       <c r="F116" s="44"/>
       <c r="G116" s="44"/>
       <c r="H116" s="44"/>
+      <c r="I116" s="71"/>
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="44"/>
@@ -33743,6 +34168,7 @@
       <c r="F117" s="44"/>
       <c r="G117" s="44"/>
       <c r="H117" s="44"/>
+      <c r="I117" s="71"/>
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="44"/>
@@ -33753,6 +34179,7 @@
       <c r="F118" s="44"/>
       <c r="G118" s="44"/>
       <c r="H118" s="44"/>
+      <c r="I118" s="71"/>
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="44"/>
@@ -33763,6 +34190,7 @@
       <c r="F119" s="44"/>
       <c r="G119" s="44"/>
       <c r="H119" s="44"/>
+      <c r="I119" s="71"/>
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="44"/>
@@ -33773,6 +34201,7 @@
       <c r="F120" s="44"/>
       <c r="G120" s="44"/>
       <c r="H120" s="44"/>
+      <c r="I120" s="71"/>
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="44"/>
@@ -33783,6 +34212,7 @@
       <c r="F121" s="44"/>
       <c r="G121" s="44"/>
       <c r="H121" s="44"/>
+      <c r="I121" s="71"/>
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A122" s="44"/>
@@ -33793,6 +34223,7 @@
       <c r="F122" s="44"/>
       <c r="G122" s="44"/>
       <c r="H122" s="44"/>
+      <c r="I122" s="71"/>
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="44"/>
@@ -33803,6 +34234,7 @@
       <c r="F123" s="44"/>
       <c r="G123" s="44"/>
       <c r="H123" s="44"/>
+      <c r="I123" s="71"/>
     </row>
     <row r="124" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="44"/>
@@ -33813,6 +34245,7 @@
       <c r="F124" s="44"/>
       <c r="G124" s="44"/>
       <c r="H124" s="44"/>
+      <c r="I124" s="71"/>
     </row>
     <row r="125" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="44"/>
@@ -33823,6 +34256,7 @@
       <c r="F125" s="44"/>
       <c r="G125" s="44"/>
       <c r="H125" s="44"/>
+      <c r="I125" s="71"/>
     </row>
     <row r="126" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="44"/>
@@ -33833,6 +34267,7 @@
       <c r="F126" s="44"/>
       <c r="G126" s="44"/>
       <c r="H126" s="44"/>
+      <c r="I126" s="71"/>
     </row>
     <row r="127" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A127" s="44"/>
@@ -33843,6 +34278,7 @@
       <c r="F127" s="44"/>
       <c r="G127" s="44"/>
       <c r="H127" s="44"/>
+      <c r="I127" s="71"/>
     </row>
     <row r="128" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="44"/>
@@ -33853,6 +34289,7 @@
       <c r="F128" s="44"/>
       <c r="G128" s="44"/>
       <c r="H128" s="44"/>
+      <c r="I128" s="71"/>
     </row>
     <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="44"/>
@@ -33863,6 +34300,7 @@
       <c r="F129" s="44"/>
       <c r="G129" s="44"/>
       <c r="H129" s="44"/>
+      <c r="I129" s="71"/>
     </row>
     <row r="130" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="44"/>
@@ -33873,6 +34311,7 @@
       <c r="F130" s="44"/>
       <c r="G130" s="44"/>
       <c r="H130" s="44"/>
+      <c r="I130" s="71"/>
     </row>
     <row r="131" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A131" s="44"/>
@@ -33883,6 +34322,7 @@
       <c r="F131" s="44"/>
       <c r="G131" s="44"/>
       <c r="H131" s="44"/>
+      <c r="I131" s="71"/>
     </row>
     <row r="132" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A132" s="44"/>
@@ -33893,6 +34333,7 @@
       <c r="F132" s="44"/>
       <c r="G132" s="44"/>
       <c r="H132" s="44"/>
+      <c r="I132" s="71"/>
     </row>
     <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="44"/>
@@ -33903,6 +34344,7 @@
       <c r="F133" s="44"/>
       <c r="G133" s="44"/>
       <c r="H133" s="44"/>
+      <c r="I133" s="71"/>
     </row>
     <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="44"/>
@@ -33913,6 +34355,7 @@
       <c r="F134" s="44"/>
       <c r="G134" s="44"/>
       <c r="H134" s="44"/>
+      <c r="I134" s="71"/>
     </row>
     <row r="135" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="44"/>
@@ -33923,6 +34366,7 @@
       <c r="F135" s="44"/>
       <c r="G135" s="44"/>
       <c r="H135" s="44"/>
+      <c r="I135" s="71"/>
     </row>
     <row r="136" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A136" s="44"/>
@@ -33933,6 +34377,7 @@
       <c r="F136" s="44"/>
       <c r="G136" s="44"/>
       <c r="H136" s="44"/>
+      <c r="I136" s="71"/>
     </row>
     <row r="137" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A137" s="44"/>
@@ -33943,6 +34388,7 @@
       <c r="F137" s="44"/>
       <c r="G137" s="44"/>
       <c r="H137" s="44"/>
+      <c r="I137" s="71"/>
     </row>
     <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="44"/>
@@ -33953,6 +34399,7 @@
       <c r="F138" s="44"/>
       <c r="G138" s="44"/>
       <c r="H138" s="44"/>
+      <c r="I138" s="71"/>
     </row>
     <row r="139" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="44"/>
@@ -33963,6 +34410,7 @@
       <c r="F139" s="44"/>
       <c r="G139" s="44"/>
       <c r="H139" s="44"/>
+      <c r="I139" s="71"/>
     </row>
     <row r="140" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A140" s="44"/>
@@ -33973,6 +34421,7 @@
       <c r="F140" s="44"/>
       <c r="G140" s="44"/>
       <c r="H140" s="44"/>
+      <c r="I140" s="71"/>
     </row>
     <row r="141" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="44"/>
@@ -33983,6 +34432,7 @@
       <c r="F141" s="44"/>
       <c r="G141" s="44"/>
       <c r="H141" s="44"/>
+      <c r="I141" s="71"/>
     </row>
     <row r="142" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A142" s="44"/>
@@ -33993,6 +34443,7 @@
       <c r="F142" s="44"/>
       <c r="G142" s="44"/>
       <c r="H142" s="44"/>
+      <c r="I142" s="71"/>
     </row>
     <row r="143" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A143" s="44"/>
@@ -34003,6 +34454,7 @@
       <c r="F143" s="44"/>
       <c r="G143" s="44"/>
       <c r="H143" s="44"/>
+      <c r="I143" s="71"/>
     </row>
     <row r="144" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="44"/>
@@ -34013,6 +34465,7 @@
       <c r="F144" s="44"/>
       <c r="G144" s="44"/>
       <c r="H144" s="44"/>
+      <c r="I144" s="71"/>
     </row>
     <row r="145" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="44"/>
@@ -34023,6 +34476,7 @@
       <c r="F145" s="44"/>
       <c r="G145" s="44"/>
       <c r="H145" s="44"/>
+      <c r="I145" s="71"/>
     </row>
     <row r="146" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A146" s="44"/>
@@ -34033,6 +34487,7 @@
       <c r="F146" s="44"/>
       <c r="G146" s="44"/>
       <c r="H146" s="44"/>
+      <c r="I146" s="71"/>
     </row>
     <row r="147" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A147" s="44"/>
@@ -34043,6 +34498,7 @@
       <c r="F147" s="44"/>
       <c r="G147" s="44"/>
       <c r="H147" s="44"/>
+      <c r="I147" s="71"/>
     </row>
     <row r="148" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A148" s="44"/>
@@ -34053,6 +34509,7 @@
       <c r="F148" s="44"/>
       <c r="G148" s="44"/>
       <c r="H148" s="44"/>
+      <c r="I148" s="71"/>
     </row>
     <row r="149" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A149" s="44"/>
@@ -34063,6 +34520,7 @@
       <c r="F149" s="44"/>
       <c r="G149" s="44"/>
       <c r="H149" s="44"/>
+      <c r="I149" s="71"/>
     </row>
     <row r="150" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A150" s="44"/>
@@ -34073,6 +34531,7 @@
       <c r="F150" s="44"/>
       <c r="G150" s="44"/>
       <c r="H150" s="44"/>
+      <c r="I150" s="71"/>
     </row>
     <row r="151" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A151" s="44"/>
@@ -34083,6 +34542,7 @@
       <c r="F151" s="44"/>
       <c r="G151" s="44"/>
       <c r="H151" s="44"/>
+      <c r="I151" s="71"/>
     </row>
     <row r="152" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A152" s="44"/>
@@ -34093,6 +34553,7 @@
       <c r="F152" s="44"/>
       <c r="G152" s="44"/>
       <c r="H152" s="44"/>
+      <c r="I152" s="71"/>
     </row>
     <row r="153" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A153" s="44"/>
@@ -34103,6 +34564,7 @@
       <c r="F153" s="44"/>
       <c r="G153" s="44"/>
       <c r="H153" s="44"/>
+      <c r="I153" s="71"/>
     </row>
     <row r="154" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A154" s="44"/>
@@ -34113,6 +34575,7 @@
       <c r="F154" s="44"/>
       <c r="G154" s="44"/>
       <c r="H154" s="44"/>
+      <c r="I154" s="71"/>
     </row>
     <row r="155" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A155" s="44"/>
@@ -34123,6 +34586,7 @@
       <c r="F155" s="44"/>
       <c r="G155" s="44"/>
       <c r="H155" s="44"/>
+      <c r="I155" s="71"/>
     </row>
     <row r="156" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A156" s="44"/>
@@ -34133,6 +34597,7 @@
       <c r="F156" s="44"/>
       <c r="G156" s="44"/>
       <c r="H156" s="44"/>
+      <c r="I156" s="71"/>
     </row>
     <row r="157" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A157" s="44"/>
@@ -34143,6 +34608,7 @@
       <c r="F157" s="44"/>
       <c r="G157" s="44"/>
       <c r="H157" s="44"/>
+      <c r="I157" s="71"/>
     </row>
     <row r="158" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A158" s="44"/>
@@ -34153,6 +34619,7 @@
       <c r="F158" s="44"/>
       <c r="G158" s="44"/>
       <c r="H158" s="44"/>
+      <c r="I158" s="71"/>
     </row>
     <row r="159" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A159" s="44"/>
@@ -34163,6 +34630,7 @@
       <c r="F159" s="44"/>
       <c r="G159" s="44"/>
       <c r="H159" s="44"/>
+      <c r="I159" s="71"/>
     </row>
     <row r="160" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A160" s="44"/>
@@ -34173,6 +34641,7 @@
       <c r="F160" s="44"/>
       <c r="G160" s="44"/>
       <c r="H160" s="44"/>
+      <c r="I160" s="71"/>
     </row>
     <row r="161" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A161" s="44"/>
@@ -34183,6 +34652,7 @@
       <c r="F161" s="44"/>
       <c r="G161" s="44"/>
       <c r="H161" s="44"/>
+      <c r="I161" s="71"/>
     </row>
     <row r="162" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A162" s="44"/>
@@ -34193,6 +34663,7 @@
       <c r="F162" s="44"/>
       <c r="G162" s="44"/>
       <c r="H162" s="44"/>
+      <c r="I162" s="71"/>
     </row>
     <row r="163" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A163" s="44"/>
@@ -34203,6 +34674,7 @@
       <c r="F163" s="44"/>
       <c r="G163" s="44"/>
       <c r="H163" s="44"/>
+      <c r="I163" s="71"/>
     </row>
     <row r="164" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A164" s="44"/>
@@ -34213,6 +34685,7 @@
       <c r="F164" s="44"/>
       <c r="G164" s="44"/>
       <c r="H164" s="44"/>
+      <c r="I164" s="71"/>
     </row>
     <row r="165" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A165" s="44"/>
@@ -34223,6 +34696,7 @@
       <c r="F165" s="44"/>
       <c r="G165" s="44"/>
       <c r="H165" s="44"/>
+      <c r="I165" s="71"/>
     </row>
     <row r="166" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A166" s="44"/>
@@ -34233,6 +34707,7 @@
       <c r="F166" s="44"/>
       <c r="G166" s="44"/>
       <c r="H166" s="44"/>
+      <c r="I166" s="71"/>
     </row>
     <row r="167" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A167" s="44"/>
@@ -34243,6 +34718,7 @@
       <c r="F167" s="44"/>
       <c r="G167" s="44"/>
       <c r="H167" s="44"/>
+      <c r="I167" s="71"/>
     </row>
     <row r="168" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A168" s="44"/>
@@ -34253,6 +34729,7 @@
       <c r="F168" s="44"/>
       <c r="G168" s="44"/>
       <c r="H168" s="44"/>
+      <c r="I168" s="71"/>
     </row>
     <row r="169" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A169" s="44"/>
@@ -34263,6 +34740,7 @@
       <c r="F169" s="44"/>
       <c r="G169" s="44"/>
       <c r="H169" s="44"/>
+      <c r="I169" s="71"/>
     </row>
     <row r="170" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A170" s="44"/>
@@ -34273,6 +34751,7 @@
       <c r="F170" s="44"/>
       <c r="G170" s="44"/>
       <c r="H170" s="44"/>
+      <c r="I170" s="71"/>
     </row>
     <row r="171" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A171" s="44"/>
@@ -34283,6 +34762,7 @@
       <c r="F171" s="44"/>
       <c r="G171" s="44"/>
       <c r="H171" s="44"/>
+      <c r="I171" s="71"/>
     </row>
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="44"/>
@@ -34293,6 +34773,7 @@
       <c r="F172" s="44"/>
       <c r="G172" s="44"/>
       <c r="H172" s="44"/>
+      <c r="I172" s="71"/>
     </row>
     <row r="173" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A173" s="44"/>
@@ -34303,6 +34784,7 @@
       <c r="F173" s="44"/>
       <c r="G173" s="44"/>
       <c r="H173" s="44"/>
+      <c r="I173" s="71"/>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A174" s="44"/>
@@ -34313,6 +34795,7 @@
       <c r="F174" s="44"/>
       <c r="G174" s="44"/>
       <c r="H174" s="44"/>
+      <c r="I174" s="71"/>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A175" s="44"/>
@@ -34323,6 +34806,7 @@
       <c r="F175" s="44"/>
       <c r="G175" s="44"/>
       <c r="H175" s="44"/>
+      <c r="I175" s="71"/>
     </row>
     <row r="176" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A176" s="44"/>
@@ -34333,6 +34817,7 @@
       <c r="F176" s="44"/>
       <c r="G176" s="44"/>
       <c r="H176" s="44"/>
+      <c r="I176" s="71"/>
     </row>
     <row r="177" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A177" s="44"/>
@@ -34343,6 +34828,7 @@
       <c r="F177" s="44"/>
       <c r="G177" s="44"/>
       <c r="H177" s="44"/>
+      <c r="I177" s="71"/>
     </row>
     <row r="178" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A178" s="44"/>
@@ -34353,6 +34839,7 @@
       <c r="F178" s="44"/>
       <c r="G178" s="44"/>
       <c r="H178" s="44"/>
+      <c r="I178" s="71"/>
     </row>
     <row r="179" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A179" s="44"/>
@@ -34363,6 +34850,7 @@
       <c r="F179" s="44"/>
       <c r="G179" s="44"/>
       <c r="H179" s="44"/>
+      <c r="I179" s="71"/>
     </row>
     <row r="180" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A180" s="44"/>
@@ -34373,6 +34861,7 @@
       <c r="F180" s="44"/>
       <c r="G180" s="44"/>
       <c r="H180" s="44"/>
+      <c r="I180" s="71"/>
     </row>
     <row r="181" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A181" s="44"/>
@@ -34383,6 +34872,7 @@
       <c r="F181" s="44"/>
       <c r="G181" s="44"/>
       <c r="H181" s="44"/>
+      <c r="I181" s="71"/>
     </row>
     <row r="182" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A182" s="44"/>
@@ -34393,6 +34883,7 @@
       <c r="F182" s="44"/>
       <c r="G182" s="44"/>
       <c r="H182" s="44"/>
+      <c r="I182" s="71"/>
     </row>
     <row r="183" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A183" s="44"/>
@@ -34403,6 +34894,7 @@
       <c r="F183" s="44"/>
       <c r="G183" s="44"/>
       <c r="H183" s="44"/>
+      <c r="I183" s="71"/>
     </row>
     <row r="184" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A184" s="44"/>
@@ -34413,6 +34905,7 @@
       <c r="F184" s="44"/>
       <c r="G184" s="44"/>
       <c r="H184" s="44"/>
+      <c r="I184" s="71"/>
     </row>
     <row r="185" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A185" s="44"/>
@@ -34423,6 +34916,7 @@
       <c r="F185" s="44"/>
       <c r="G185" s="44"/>
       <c r="H185" s="44"/>
+      <c r="I185" s="71"/>
     </row>
     <row r="186" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A186" s="44"/>
@@ -34433,6 +34927,7 @@
       <c r="F186" s="44"/>
       <c r="G186" s="44"/>
       <c r="H186" s="44"/>
+      <c r="I186" s="71"/>
     </row>
     <row r="187" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A187" s="44"/>
@@ -34443,6 +34938,7 @@
       <c r="F187" s="44"/>
       <c r="G187" s="44"/>
       <c r="H187" s="44"/>
+      <c r="I187" s="71"/>
     </row>
     <row r="188" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A188" s="44"/>
@@ -34453,6 +34949,7 @@
       <c r="F188" s="44"/>
       <c r="G188" s="44"/>
       <c r="H188" s="44"/>
+      <c r="I188" s="71"/>
     </row>
     <row r="189" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A189" s="44"/>
@@ -34463,6 +34960,7 @@
       <c r="F189" s="44"/>
       <c r="G189" s="44"/>
       <c r="H189" s="44"/>
+      <c r="I189" s="71"/>
     </row>
     <row r="190" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A190" s="44"/>
@@ -34473,6 +34971,7 @@
       <c r="F190" s="44"/>
       <c r="G190" s="44"/>
       <c r="H190" s="44"/>
+      <c r="I190" s="71"/>
     </row>
     <row r="191" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A191" s="44"/>
@@ -34483,6 +34982,7 @@
       <c r="F191" s="44"/>
       <c r="G191" s="44"/>
       <c r="H191" s="44"/>
+      <c r="I191" s="71"/>
     </row>
     <row r="192" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A192" s="44"/>
@@ -34493,6 +34993,7 @@
       <c r="F192" s="44"/>
       <c r="G192" s="44"/>
       <c r="H192" s="44"/>
+      <c r="I192" s="71"/>
     </row>
     <row r="193" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A193" s="44"/>
@@ -34503,6 +35004,7 @@
       <c r="F193" s="44"/>
       <c r="G193" s="44"/>
       <c r="H193" s="44"/>
+      <c r="I193" s="71"/>
     </row>
     <row r="194" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A194" s="44"/>
@@ -34513,6 +35015,7 @@
       <c r="F194" s="44"/>
       <c r="G194" s="44"/>
       <c r="H194" s="44"/>
+      <c r="I194" s="71"/>
     </row>
     <row r="195" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A195" s="44"/>
@@ -34523,6 +35026,7 @@
       <c r="F195" s="44"/>
       <c r="G195" s="44"/>
       <c r="H195" s="44"/>
+      <c r="I195" s="71"/>
     </row>
     <row r="196" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A196" s="44"/>
@@ -34533,6 +35037,7 @@
       <c r="F196" s="44"/>
       <c r="G196" s="44"/>
       <c r="H196" s="44"/>
+      <c r="I196" s="71"/>
     </row>
     <row r="197" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A197" s="44"/>
@@ -34543,6 +35048,7 @@
       <c r="F197" s="44"/>
       <c r="G197" s="44"/>
       <c r="H197" s="44"/>
+      <c r="I197" s="71"/>
     </row>
     <row r="198" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A198" s="44"/>
@@ -34553,6 +35059,7 @@
       <c r="F198" s="44"/>
       <c r="G198" s="44"/>
       <c r="H198" s="44"/>
+      <c r="I198" s="71"/>
     </row>
     <row r="199" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A199" s="44"/>
@@ -34563,6 +35070,7 @@
       <c r="F199" s="44"/>
       <c r="G199" s="44"/>
       <c r="H199" s="44"/>
+      <c r="I199" s="71"/>
     </row>
     <row r="200" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A200" s="44"/>
@@ -34573,6 +35081,7 @@
       <c r="F200" s="44"/>
       <c r="G200" s="44"/>
       <c r="H200" s="44"/>
+      <c r="I200" s="71"/>
     </row>
     <row r="201" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A201" s="44"/>
@@ -34583,6 +35092,7 @@
       <c r="F201" s="44"/>
       <c r="G201" s="44"/>
       <c r="H201" s="44"/>
+      <c r="I201" s="71"/>
     </row>
     <row r="202" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A202" s="44"/>
@@ -34593,6 +35103,7 @@
       <c r="F202" s="44"/>
       <c r="G202" s="44"/>
       <c r="H202" s="44"/>
+      <c r="I202" s="71"/>
     </row>
     <row r="203" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A203" s="44"/>
@@ -34603,6 +35114,7 @@
       <c r="F203" s="44"/>
       <c r="G203" s="44"/>
       <c r="H203" s="44"/>
+      <c r="I203" s="71"/>
     </row>
     <row r="204" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A204" s="44"/>
@@ -34613,6 +35125,7 @@
       <c r="F204" s="44"/>
       <c r="G204" s="44"/>
       <c r="H204" s="44"/>
+      <c r="I204" s="71"/>
     </row>
     <row r="205" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A205" s="53"/>
@@ -34623,12 +35136,13 @@
       <c r="F205" s="53"/>
       <c r="G205" s="53"/>
       <c r="H205" s="53"/>
+      <c r="I205" s="72"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A4:I4"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E205">
     <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="No" dxfId="15">
@@ -34638,10 +35152,14 @@
       <formula>NOT(ISERROR(SEARCH("Yes",E6)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E6:E205" type="list">
       <formula1>"Yes,No,Partial"</formula1>
       <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I6:I205" type="whole">
+      <formula1>0</formula1>
+      <formula2>1440</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -34673,42 +35191,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>152</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -34722,98 +35240,98 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>153</v>
+        <v>174</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>155</v>
+        <v>176</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>156</v>
-      </c>
-      <c r="B5" s="68" t="n">
+        <v>177</v>
+      </c>
+      <c r="B5" s="73" t="n">
         <v>0.25</v>
       </c>
-      <c r="C5" s="68" t="n">
+      <c r="C5" s="73" t="n">
         <v>1.25</v>
       </c>
-      <c r="D5" s="68" t="n">
+      <c r="D5" s="73" t="n">
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>157</v>
+        <v>178</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>158</v>
+        <v>179</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>159</v>
-      </c>
-      <c r="B6" s="68" t="n">
+        <v>180</v>
+      </c>
+      <c r="B6" s="73" t="n">
         <v>0.25</v>
       </c>
-      <c r="C6" s="68" t="n">
+      <c r="C6" s="73" t="n">
         <v>0.5</v>
       </c>
-      <c r="D6" s="68" t="n">
+      <c r="D6" s="73" t="n">
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>160</v>
+        <v>181</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="68" t="n">
+        <v>183</v>
+      </c>
+      <c r="B7" s="73" t="n">
         <v>0.1</v>
       </c>
-      <c r="C7" s="68" t="n">
+      <c r="C7" s="73" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="68" t="n">
+      <c r="D7" s="73" t="n">
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>163</v>
+        <v>184</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>164</v>
+        <v>185</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>165</v>
-      </c>
-      <c r="B8" s="68" t="n">
+        <v>186</v>
+      </c>
+      <c r="B8" s="73" t="n">
         <v>0.01</v>
       </c>
-      <c r="C8" s="68" t="n">
+      <c r="C8" s="73" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="68" t="n">
+      <c r="D8" s="73" t="n">
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>166</v>
+        <v>187</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>167</v>
+        <v>188</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>168</v>
+        <v>189</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -34822,7 +35340,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>169</v>
+        <v>190</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -34832,86 +35350,86 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="69" t="s">
-        <v>170</v>
-      </c>
-      <c r="B11" s="69" t="s">
-        <v>171</v>
-      </c>
-      <c r="C11" s="69" t="s">
-        <v>172</v>
-      </c>
-      <c r="D11" s="69" t="s">
-        <v>144</v>
-      </c>
-      <c r="E11" s="69" t="s">
-        <v>173</v>
-      </c>
-      <c r="F11" s="69" t="s">
-        <v>174</v>
+      <c r="A11" s="74" t="s">
+        <v>191</v>
+      </c>
+      <c r="B11" s="74" t="s">
+        <v>192</v>
+      </c>
+      <c r="C11" s="74" t="s">
+        <v>193</v>
+      </c>
+      <c r="D11" s="74" t="s">
+        <v>146</v>
+      </c>
+      <c r="E11" s="74" t="s">
+        <v>194</v>
+      </c>
+      <c r="F11" s="74" t="s">
+        <v>195</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="69" t="s">
-        <v>175</v>
-      </c>
-      <c r="B12" s="69" t="s">
-        <v>176</v>
-      </c>
-      <c r="C12" s="69" t="s">
-        <v>177</v>
-      </c>
-      <c r="D12" s="69" t="s">
-        <v>178</v>
-      </c>
-      <c r="E12" s="69" t="s">
-        <v>179</v>
-      </c>
-      <c r="F12" s="69" t="s">
-        <v>180</v>
+      <c r="A12" s="74" t="s">
+        <v>196</v>
+      </c>
+      <c r="B12" s="74" t="s">
+        <v>197</v>
+      </c>
+      <c r="C12" s="74" t="s">
+        <v>198</v>
+      </c>
+      <c r="D12" s="74" t="s">
+        <v>199</v>
+      </c>
+      <c r="E12" s="74" t="s">
+        <v>200</v>
+      </c>
+      <c r="F12" s="74" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="69" t="s">
-        <v>181</v>
-      </c>
-      <c r="B13" s="69"/>
-      <c r="C13" s="69" t="s">
-        <v>182</v>
-      </c>
-      <c r="D13" s="69"/>
-      <c r="E13" s="69" t="s">
-        <v>183</v>
-      </c>
-      <c r="F13" s="69"/>
+      <c r="A13" s="74" t="s">
+        <v>202</v>
+      </c>
+      <c r="B13" s="74"/>
+      <c r="C13" s="74" t="s">
+        <v>203</v>
+      </c>
+      <c r="D13" s="74"/>
+      <c r="E13" s="74" t="s">
+        <v>204</v>
+      </c>
+      <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="69" t="s">
-        <v>184</v>
-      </c>
-      <c r="B14" s="69"/>
-      <c r="C14" s="69" t="s">
-        <v>185</v>
-      </c>
-      <c r="D14" s="69"/>
-      <c r="E14" s="69" t="s">
-        <v>186</v>
-      </c>
-      <c r="F14" s="69"/>
+      <c r="A14" s="74" t="s">
+        <v>205</v>
+      </c>
+      <c r="B14" s="74"/>
+      <c r="C14" s="74" t="s">
+        <v>206</v>
+      </c>
+      <c r="D14" s="74"/>
+      <c r="E14" s="74" t="s">
+        <v>207</v>
+      </c>
+      <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="69" t="s">
-        <v>187</v>
-      </c>
-      <c r="B15" s="69"/>
-      <c r="C15" s="69" t="s">
-        <v>188</v>
-      </c>
-      <c r="D15" s="69"/>
-      <c r="E15" s="69" t="s">
-        <v>189</v>
-      </c>
-      <c r="F15" s="69"/>
+      <c r="A15" s="74" t="s">
+        <v>208</v>
+      </c>
+      <c r="B15" s="74"/>
+      <c r="C15" s="74" t="s">
+        <v>209</v>
+      </c>
+      <c r="D15" s="74"/>
+      <c r="E15" s="74" t="s">
+        <v>210</v>
+      </c>
+      <c r="F15" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -34948,106 +35466,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>191</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>192</v>
+        <v>213</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>193</v>
+        <v>214</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>195</v>
+        <v>216</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>196</v>
+        <v>217</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>197</v>
+        <v>218</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>198</v>
+        <v>219</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>199</v>
+        <v>220</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>200</v>
+        <v>221</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35055,25 +35573,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>202</v>
+        <v>223</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>204</v>
+        <v>225</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>205</v>
+        <v>226</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>206</v>
+        <v>227</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>207</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35081,25 +35599,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>208</v>
+        <v>229</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>209</v>
+        <v>230</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>212</v>
+        <v>233</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>213</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35107,25 +35625,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>214</v>
+        <v>235</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>215</v>
+        <v>236</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>216</v>
+        <v>237</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>217</v>
+        <v>238</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35133,25 +35651,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>220</v>
+        <v>241</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>221</v>
+        <v>242</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>222</v>
+        <v>243</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>225</v>
+        <v>246</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>226</v>
+        <v>247</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35159,65 +35677,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>227</v>
+        <v>248</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>228</v>
+        <v>249</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>229</v>
+        <v>250</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>223</v>
+        <v>244</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>224</v>
+        <v>245</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>230</v>
+        <v>251</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>231</v>
+        <v>252</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>232</v>
+        <v>253</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>233</v>
+        <v>254</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>234</v>
+        <v>255</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>235</v>
+        <v>256</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>194</v>
+        <v>215</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35225,109 +35743,109 @@
       <c r="H13" s="34"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="70" t="s">
-        <v>236</v>
-      </c>
-      <c r="B14" s="71" t="s">
-        <v>237</v>
-      </c>
-      <c r="C14" s="71" t="s">
-        <v>238</v>
-      </c>
-      <c r="D14" s="71" t="s">
-        <v>239</v>
-      </c>
-      <c r="E14" s="71"/>
-      <c r="F14" s="71"/>
-      <c r="G14" s="71"/>
-      <c r="H14" s="71"/>
+      <c r="A14" s="75" t="s">
+        <v>257</v>
+      </c>
+      <c r="B14" s="76" t="s">
+        <v>258</v>
+      </c>
+      <c r="C14" s="76" t="s">
+        <v>259</v>
+      </c>
+      <c r="D14" s="76" t="s">
+        <v>260</v>
+      </c>
+      <c r="E14" s="76"/>
+      <c r="F14" s="76"/>
+      <c r="G14" s="76"/>
+      <c r="H14" s="76"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="72" t="s">
-        <v>240</v>
-      </c>
-      <c r="B15" s="71" t="s">
-        <v>241</v>
-      </c>
-      <c r="C15" s="71" t="s">
+      <c r="A15" s="77" t="s">
+        <v>261</v>
+      </c>
+      <c r="B15" s="76" t="s">
+        <v>262</v>
+      </c>
+      <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
-      <c r="D15" s="71" t="s">
-        <v>242</v>
-      </c>
-      <c r="E15" s="71"/>
-      <c r="F15" s="71"/>
-      <c r="G15" s="71"/>
-      <c r="H15" s="71"/>
+      <c r="D15" s="76" t="s">
+        <v>263</v>
+      </c>
+      <c r="E15" s="76"/>
+      <c r="F15" s="76"/>
+      <c r="G15" s="76"/>
+      <c r="H15" s="76"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="73" t="s">
-        <v>243</v>
-      </c>
-      <c r="B16" s="71" t="s">
-        <v>244</v>
-      </c>
-      <c r="C16" s="71" t="s">
-        <v>245</v>
-      </c>
-      <c r="D16" s="71" t="s">
-        <v>246</v>
-      </c>
-      <c r="E16" s="71"/>
-      <c r="F16" s="71"/>
-      <c r="G16" s="71"/>
-      <c r="H16" s="71"/>
+      <c r="A16" s="78" t="s">
+        <v>264</v>
+      </c>
+      <c r="B16" s="76" t="s">
+        <v>265</v>
+      </c>
+      <c r="C16" s="76" t="s">
+        <v>266</v>
+      </c>
+      <c r="D16" s="76" t="s">
+        <v>267</v>
+      </c>
+      <c r="E16" s="76"/>
+      <c r="F16" s="76"/>
+      <c r="G16" s="76"/>
+      <c r="H16" s="76"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="74" t="s">
-        <v>247</v>
-      </c>
-      <c r="B17" s="71" t="s">
-        <v>248</v>
-      </c>
-      <c r="C17" s="71" t="s">
-        <v>249</v>
-      </c>
-      <c r="D17" s="71" t="s">
-        <v>250</v>
-      </c>
-      <c r="E17" s="71"/>
-      <c r="F17" s="71"/>
-      <c r="G17" s="71"/>
-      <c r="H17" s="71"/>
+      <c r="A17" s="79" t="s">
+        <v>268</v>
+      </c>
+      <c r="B17" s="76" t="s">
+        <v>269</v>
+      </c>
+      <c r="C17" s="76" t="s">
+        <v>270</v>
+      </c>
+      <c r="D17" s="76" t="s">
+        <v>271</v>
+      </c>
+      <c r="E17" s="76"/>
+      <c r="F17" s="76"/>
+      <c r="G17" s="76"/>
+      <c r="H17" s="76"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>252</v>
+        <v>273</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -35337,151 +35855,151 @@
       <c r="H20" s="34"/>
     </row>
     <row r="21" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="71" t="s">
+      <c r="A21" s="76" t="s">
         <v>96</v>
       </c>
-      <c r="B21" s="71" t="s">
-        <v>254</v>
-      </c>
-      <c r="C21" s="71"/>
-      <c r="D21" s="71"/>
-      <c r="E21" s="71"/>
-      <c r="F21" s="71"/>
-      <c r="G21" s="71"/>
-      <c r="H21" s="71"/>
+      <c r="B21" s="76" t="s">
+        <v>275</v>
+      </c>
+      <c r="C21" s="76"/>
+      <c r="D21" s="76"/>
+      <c r="E21" s="76"/>
+      <c r="F21" s="76"/>
+      <c r="G21" s="76"/>
+      <c r="H21" s="76"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="71" t="s">
+      <c r="A22" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="71" t="s">
-        <v>255</v>
-      </c>
-      <c r="C22" s="71"/>
-      <c r="D22" s="71"/>
-      <c r="E22" s="71"/>
-      <c r="F22" s="71"/>
-      <c r="G22" s="71"/>
-      <c r="H22" s="71"/>
+      <c r="B22" s="76" t="s">
+        <v>276</v>
+      </c>
+      <c r="C22" s="76"/>
+      <c r="D22" s="76"/>
+      <c r="E22" s="76"/>
+      <c r="F22" s="76"/>
+      <c r="G22" s="76"/>
+      <c r="H22" s="76"/>
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="71" t="s">
-        <v>256</v>
-      </c>
-      <c r="B23" s="71" t="s">
-        <v>257</v>
-      </c>
-      <c r="C23" s="71"/>
-      <c r="D23" s="71"/>
-      <c r="E23" s="71"/>
-      <c r="F23" s="71"/>
-      <c r="G23" s="71"/>
-      <c r="H23" s="71"/>
+      <c r="A23" s="76" t="s">
+        <v>277</v>
+      </c>
+      <c r="B23" s="76" t="s">
+        <v>278</v>
+      </c>
+      <c r="C23" s="76"/>
+      <c r="D23" s="76"/>
+      <c r="E23" s="76"/>
+      <c r="F23" s="76"/>
+      <c r="G23" s="76"/>
+      <c r="H23" s="76"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="71" t="s">
+      <c r="A24" s="76" t="s">
         <v>98</v>
       </c>
-      <c r="B24" s="71" t="s">
-        <v>258</v>
-      </c>
-      <c r="C24" s="71"/>
-      <c r="D24" s="71"/>
-      <c r="E24" s="71"/>
-      <c r="F24" s="71"/>
-      <c r="G24" s="71"/>
-      <c r="H24" s="71"/>
+      <c r="B24" s="76" t="s">
+        <v>279</v>
+      </c>
+      <c r="C24" s="76"/>
+      <c r="D24" s="76"/>
+      <c r="E24" s="76"/>
+      <c r="F24" s="76"/>
+      <c r="G24" s="76"/>
+      <c r="H24" s="76"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="71" t="s">
+      <c r="A25" s="76" t="s">
         <v>109</v>
       </c>
-      <c r="B25" s="71" t="s">
-        <v>259</v>
-      </c>
-      <c r="C25" s="71"/>
-      <c r="D25" s="71"/>
-      <c r="E25" s="71"/>
-      <c r="F25" s="71"/>
-      <c r="G25" s="71"/>
-      <c r="H25" s="71"/>
+      <c r="B25" s="76" t="s">
+        <v>280</v>
+      </c>
+      <c r="C25" s="76"/>
+      <c r="D25" s="76"/>
+      <c r="E25" s="76"/>
+      <c r="F25" s="76"/>
+      <c r="G25" s="76"/>
+      <c r="H25" s="76"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 2 Part C
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="729" uniqueCount="282">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="283">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -543,6 +543,9 @@
   </si>
   <si>
     <t xml:space="preserve">P&amp;L from fills</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planned risk and costs</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -2448,7 +2451,7 @@
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33073,13 +33076,25 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="44"/>
       <c r="B18" s="45"/>
-      <c r="C18" s="48"/>
-      <c r="D18" s="44"/>
-      <c r="E18" s="44"/>
-      <c r="F18" s="44"/>
+      <c r="C18" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="44" t="s">
+        <v>152</v>
+      </c>
+      <c r="E18" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F18" s="44" t="s">
+        <v>172</v>
+      </c>
       <c r="G18" s="44"/>
-      <c r="H18" s="44"/>
-      <c r="I18" s="71"/>
+      <c r="H18" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="I18" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="44"/>
@@ -35191,42 +35206,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35240,18 +35255,18 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B5" s="73" t="n">
         <v>0.25</v>
@@ -35263,15 +35278,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B6" s="73" t="n">
         <v>0.25</v>
@@ -35283,15 +35298,15 @@
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B7" s="73" t="n">
         <v>0.1</v>
@@ -35303,15 +35318,15 @@
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B8" s="73" t="n">
         <v>0.01</v>
@@ -35323,15 +35338,15 @@
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -35340,7 +35355,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -35351,83 +35366,83 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="74" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D11" s="74" t="s">
         <v>146</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="74" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B12" s="74" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C12" s="74" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D12" s="74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F12" s="74" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="74" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B13" s="74"/>
       <c r="C13" s="74" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D13" s="74"/>
       <c r="E13" s="74" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="74" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B14" s="74"/>
       <c r="C14" s="74" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D14" s="74"/>
       <c r="E14" s="74" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="74" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="74" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="D15" s="74"/>
       <c r="E15" s="74" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F15" s="74"/>
     </row>
@@ -35466,106 +35481,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35573,25 +35588,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35599,25 +35614,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35625,25 +35640,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35651,25 +35666,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35677,65 +35692,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35744,16 +35759,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="75" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B14" s="76" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D14" s="76" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="E14" s="76"/>
       <c r="F14" s="76"/>
@@ -35762,16 +35777,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="77" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B15" s="76" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="E15" s="76"/>
       <c r="F15" s="76"/>
@@ -35780,16 +35795,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="78" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B16" s="76" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D16" s="76" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="E16" s="76"/>
       <c r="F16" s="76"/>
@@ -35798,16 +35813,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="79" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E17" s="76"/>
       <c r="F17" s="76"/>
@@ -35816,36 +35831,36 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -35859,7 +35874,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="76" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="76"/>
@@ -35873,7 +35888,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="76" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C22" s="76"/>
       <c r="D22" s="76"/>
@@ -35884,10 +35899,10 @@
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="C23" s="76"/>
       <c r="D23" s="76"/>
@@ -35901,7 +35916,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="76" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C24" s="76"/>
       <c r="D24" s="76"/>
@@ -35915,7 +35930,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="76" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C25" s="76"/>
       <c r="D25" s="76"/>
@@ -35926,80 +35941,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 2 Part D
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="737" uniqueCount="284">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -546,6 +546,9 @@
   </si>
   <si>
     <t xml:space="preserve">Planned risk and costs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spread and cost</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -2451,7 +2454,7 @@
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>11.5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33099,13 +33102,25 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="44"/>
       <c r="B19" s="45"/>
-      <c r="C19" s="48"/>
-      <c r="D19" s="44"/>
-      <c r="E19" s="44"/>
-      <c r="F19" s="44"/>
+      <c r="C19" s="48" t="n">
+        <v>2</v>
+      </c>
+      <c r="D19" s="44" t="s">
+        <v>154</v>
+      </c>
+      <c r="E19" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F19" s="44" t="s">
+        <v>173</v>
+      </c>
       <c r="G19" s="44"/>
-      <c r="H19" s="44"/>
-      <c r="I19" s="71"/>
+      <c r="H19" s="44" t="s">
+        <v>169</v>
+      </c>
+      <c r="I19" s="71" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="44"/>
@@ -35206,42 +35221,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35255,18 +35270,18 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B5" s="73" t="n">
         <v>0.25</v>
@@ -35278,15 +35293,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B6" s="73" t="n">
         <v>0.25</v>
@@ -35298,15 +35313,15 @@
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B7" s="73" t="n">
         <v>0.1</v>
@@ -35318,15 +35333,15 @@
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B8" s="73" t="n">
         <v>0.01</v>
@@ -35338,15 +35353,15 @@
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -35355,7 +35370,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -35366,83 +35381,83 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="74" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D11" s="74" t="s">
         <v>146</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="74" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B12" s="74" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="C12" s="74" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="D12" s="74" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F12" s="74" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="74" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B13" s="74"/>
       <c r="C13" s="74" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D13" s="74"/>
       <c r="E13" s="74" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="74" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B14" s="74"/>
       <c r="C14" s="74" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="D14" s="74"/>
       <c r="E14" s="74" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="74" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="74" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D15" s="74"/>
       <c r="E15" s="74" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F15" s="74"/>
     </row>
@@ -35481,106 +35496,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35588,25 +35603,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35614,25 +35629,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35640,25 +35655,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35666,25 +35681,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35692,65 +35707,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35759,16 +35774,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="75" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B14" s="76" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D14" s="76" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="E14" s="76"/>
       <c r="F14" s="76"/>
@@ -35777,16 +35792,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="77" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B15" s="76" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E15" s="76"/>
       <c r="F15" s="76"/>
@@ -35795,16 +35810,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="78" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B16" s="76" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D16" s="76" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="E16" s="76"/>
       <c r="F16" s="76"/>
@@ -35813,16 +35828,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="79" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E17" s="76"/>
       <c r="F17" s="76"/>
@@ -35831,36 +35846,36 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -35874,7 +35889,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="76" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="76"/>
@@ -35888,7 +35903,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="76" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C22" s="76"/>
       <c r="D22" s="76"/>
@@ -35899,10 +35914,10 @@
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C23" s="76"/>
       <c r="D23" s="76"/>
@@ -35916,7 +35931,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="76" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C24" s="76"/>
       <c r="D24" s="76"/>
@@ -35930,7 +35945,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="76" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C25" s="76"/>
       <c r="D25" s="76"/>
@@ -35941,80 +35956,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 3 add log time for Part A and B
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="754" uniqueCount="296">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="758" uniqueCount="299">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -585,6 +585,15 @@
   </si>
   <si>
     <t xml:space="preserve">Part 7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Part A and B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concensus, actual for MES MGC MCL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See week 3 assignment</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -2490,7 +2499,7 @@
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>15.6666666666667</v>
+        <v>16.6666666666667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33260,13 +33269,25 @@
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="44"/>
       <c r="B23" s="45"/>
-      <c r="C23" s="48"/>
-      <c r="D23" s="44"/>
-      <c r="E23" s="44"/>
-      <c r="F23" s="44"/>
+      <c r="C23" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D23" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="E23" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F23" s="44" t="s">
+        <v>187</v>
+      </c>
       <c r="G23" s="44"/>
-      <c r="H23" s="44"/>
-      <c r="I23" s="71"/>
+      <c r="H23" s="44" t="s">
+        <v>188</v>
+      </c>
+      <c r="I23" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="44"/>
@@ -35323,42 +35344,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35372,18 +35393,18 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B5" s="73" t="n">
         <v>0.25</v>
@@ -35395,15 +35416,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B6" s="73" t="n">
         <v>0.25</v>
@@ -35415,15 +35436,15 @@
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B7" s="73" t="n">
         <v>0.1</v>
@@ -35435,15 +35456,15 @@
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B8" s="73" t="n">
         <v>0.01</v>
@@ -35455,15 +35476,15 @@
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -35472,7 +35493,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -35483,83 +35504,83 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="74" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D11" s="74" t="s">
         <v>146</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="74" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B12" s="74" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="C12" s="74" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="D12" s="74" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F12" s="74" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="74" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B13" s="74"/>
       <c r="C13" s="74" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="D13" s="74"/>
       <c r="E13" s="74" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="74" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B14" s="74"/>
       <c r="C14" s="74" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="D14" s="74"/>
       <c r="E14" s="74" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="74" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="74" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D15" s="74"/>
       <c r="E15" s="74" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F15" s="74"/>
     </row>
@@ -35598,106 +35619,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35705,25 +35726,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35731,25 +35752,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35757,25 +35778,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35783,25 +35804,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35809,65 +35830,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
+        <v>265</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>266</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>267</v>
+      </c>
+      <c r="E10" s="24" t="s">
+        <v>261</v>
+      </c>
+      <c r="F10" s="24" t="s">
         <v>262</v>
       </c>
-      <c r="C10" s="24" t="s">
-        <v>263</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>264</v>
-      </c>
-      <c r="E10" s="24" t="s">
-        <v>258</v>
-      </c>
-      <c r="F10" s="24" t="s">
-        <v>259</v>
-      </c>
       <c r="G10" s="24" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35876,16 +35897,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="75" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B14" s="76" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D14" s="76" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="E14" s="76"/>
       <c r="F14" s="76"/>
@@ -35894,16 +35915,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="77" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B15" s="76" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="E15" s="76"/>
       <c r="F15" s="76"/>
@@ -35912,16 +35933,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="78" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B16" s="76" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D16" s="76" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="E16" s="76"/>
       <c r="F16" s="76"/>
@@ -35930,16 +35951,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="79" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="E17" s="76"/>
       <c r="F17" s="76"/>
@@ -35948,36 +35969,36 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -35991,7 +36012,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="76" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="76"/>
@@ -36005,7 +36026,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="76" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="C22" s="76"/>
       <c r="D22" s="76"/>
@@ -36016,10 +36037,10 @@
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="C23" s="76"/>
       <c r="D23" s="76"/>
@@ -36033,7 +36054,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="76" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="C24" s="76"/>
       <c r="D24" s="76"/>
@@ -36047,7 +36068,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="76" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="C25" s="76"/>
       <c r="D25" s="76"/>
@@ -36058,80 +36079,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 3 Case 2 MES
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="302">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="308">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -587,6 +587,9 @@
     <t xml:space="preserve">Part 7</t>
   </si>
   <si>
+    <t xml:space="preserve">W03-1</t>
+  </si>
+  <si>
     <t xml:space="preserve">Part A and B</t>
   </si>
   <si>
@@ -596,6 +599,9 @@
     <t xml:space="preserve">See week 3 assignment</t>
   </si>
   <si>
+    <t xml:space="preserve">W03-2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fiche MES CASE 1</t>
   </si>
   <si>
@@ -603,6 +609,18 @@
   </si>
   <si>
     <t xml:space="preserve">See research week 3 01-mes.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W03-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche MES CASE 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donnée de l’emploi au États-Unis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See research week 3 02-mes.md</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -2508,7 +2526,7 @@
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>17.6666666666667</v>
+        <v>18.6666666666667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33276,61 +33294,85 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="44"/>
-      <c r="B23" s="45"/>
+      <c r="A23" s="44" t="s">
+        <v>186</v>
+      </c>
+      <c r="B23" s="45" t="n">
+        <v>46293</v>
+      </c>
       <c r="C23" s="48" t="n">
         <v>3</v>
       </c>
       <c r="D23" s="44" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="E23" s="44" t="s">
         <v>146</v>
       </c>
       <c r="F23" s="44" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G23" s="44"/>
       <c r="H23" s="44" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I23" s="71" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="44"/>
-      <c r="B24" s="45"/>
+      <c r="A24" s="44" t="s">
+        <v>190</v>
+      </c>
+      <c r="B24" s="45" t="n">
+        <v>46294</v>
+      </c>
       <c r="C24" s="48" t="n">
         <v>3</v>
       </c>
       <c r="D24" s="44" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="E24" s="44" t="s">
         <v>146</v>
       </c>
       <c r="F24" s="44" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G24" s="44"/>
       <c r="H24" s="44" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="I24" s="71" t="n">
         <v>60</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="44"/>
-      <c r="B25" s="45"/>
-      <c r="C25" s="48"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
+      <c r="A25" s="44" t="s">
+        <v>194</v>
+      </c>
+      <c r="B25" s="45" t="n">
+        <v>46295</v>
+      </c>
+      <c r="C25" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D25" s="44" t="s">
+        <v>195</v>
+      </c>
+      <c r="E25" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F25" s="44" t="s">
+        <v>196</v>
+      </c>
       <c r="G25" s="44"/>
-      <c r="H25" s="44"/>
-      <c r="I25" s="71"/>
+      <c r="H25" s="44" t="s">
+        <v>197</v>
+      </c>
+      <c r="I25" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="44"/>
@@ -35365,42 +35407,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35414,18 +35456,18 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B5" s="73" t="n">
         <v>0.25</v>
@@ -35437,15 +35479,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="B6" s="73" t="n">
         <v>0.25</v>
@@ -35457,15 +35499,15 @@
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="B7" s="73" t="n">
         <v>0.1</v>
@@ -35477,15 +35519,15 @@
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="B8" s="73" t="n">
         <v>0.01</v>
@@ -35497,15 +35539,15 @@
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -35514,7 +35556,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -35525,83 +35567,83 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="74" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="D11" s="74" t="s">
         <v>146</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="74" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="B12" s="74" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="C12" s="74" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="D12" s="74" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="F12" s="74" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="74" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B13" s="74"/>
       <c r="C13" s="74" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="D13" s="74"/>
       <c r="E13" s="74" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="74" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="B14" s="74"/>
       <c r="C14" s="74" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="D14" s="74"/>
       <c r="E14" s="74" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="74" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="74" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="D15" s="74"/>
       <c r="E15" s="74" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="F15" s="74"/>
     </row>
@@ -35640,106 +35682,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35747,25 +35789,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35773,25 +35815,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35799,25 +35841,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35825,25 +35867,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35851,65 +35893,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="D10" s="24" t="s">
+        <v>276</v>
+      </c>
+      <c r="E10" s="24" t="s">
         <v>270</v>
       </c>
-      <c r="E10" s="24" t="s">
-        <v>264</v>
-      </c>
       <c r="F10" s="24" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35918,16 +35960,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="75" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="B14" s="76" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="D14" s="76" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
       <c r="E14" s="76"/>
       <c r="F14" s="76"/>
@@ -35936,16 +35978,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="77" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="B15" s="76" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E15" s="76"/>
       <c r="F15" s="76"/>
@@ -35954,16 +35996,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="78" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="B16" s="76" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="D16" s="76" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="E16" s="76"/>
       <c r="F16" s="76"/>
@@ -35972,16 +36014,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="79" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="E17" s="76"/>
       <c r="F17" s="76"/>
@@ -35990,36 +36032,36 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -36033,7 +36075,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="76" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="76"/>
@@ -36047,7 +36089,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="76" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="C22" s="76"/>
       <c r="D22" s="76"/>
@@ -36058,10 +36100,10 @@
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
       <c r="C23" s="76"/>
       <c r="D23" s="76"/>
@@ -36075,7 +36117,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="76" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="C24" s="76"/>
       <c r="D24" s="76"/>
@@ -36089,7 +36131,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="76" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="C25" s="76"/>
       <c r="D25" s="76"/>
@@ -36100,80 +36142,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Week 3 case 3 and 4
</commit_message>
<xml_diff>
--- a/journal/trading-journal.xlsx
+++ b/journal/trading-journal.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="769" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="779" uniqueCount="316">
   <si>
     <t xml:space="preserve">Futures Trading Academy — Journal Dashboard</t>
   </si>
@@ -621,6 +621,30 @@
   </si>
   <si>
     <t xml:space="preserve">See research week 3 02-mes.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W03-4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche MES CASE 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donnée des PPI au États-Unis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See research week 3 03-mes.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">W03-5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fiche MES CASE 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Donnée de Taux de la fed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">See research week 3 04-mgc.md</t>
   </si>
   <si>
     <t xml:space="preserve">Reference Lists</t>
@@ -2526,7 +2550,7 @@
       </c>
       <c r="H10" s="16" t="n">
         <f aca="false">SUMIFS('Study Log'!$I$6:$I$205,'Study Log'!$A$6:$A$205,"&lt;&gt;EXAMPLE-001")/60</f>
-        <v>18.6666666666667</v>
+        <v>20.1666666666667</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -33375,26 +33399,58 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="44"/>
-      <c r="B26" s="45"/>
-      <c r="C26" s="48"/>
-      <c r="D26" s="44"/>
-      <c r="E26" s="44"/>
-      <c r="F26" s="44"/>
+      <c r="A26" s="44" t="s">
+        <v>198</v>
+      </c>
+      <c r="B26" s="45" t="n">
+        <v>46300</v>
+      </c>
+      <c r="C26" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D26" s="44" t="s">
+        <v>199</v>
+      </c>
+      <c r="E26" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F26" s="44" t="s">
+        <v>200</v>
+      </c>
       <c r="G26" s="44"/>
-      <c r="H26" s="44"/>
-      <c r="I26" s="71"/>
+      <c r="H26" s="44" t="s">
+        <v>201</v>
+      </c>
+      <c r="I26" s="71" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="44"/>
-      <c r="B27" s="45"/>
-      <c r="C27" s="48"/>
-      <c r="D27" s="44"/>
-      <c r="E27" s="44"/>
-      <c r="F27" s="44"/>
+      <c r="A27" s="44" t="s">
+        <v>202</v>
+      </c>
+      <c r="B27" s="45" t="n">
+        <v>46301</v>
+      </c>
+      <c r="C27" s="48" t="n">
+        <v>3</v>
+      </c>
+      <c r="D27" s="44" t="s">
+        <v>203</v>
+      </c>
+      <c r="E27" s="44" t="s">
+        <v>146</v>
+      </c>
+      <c r="F27" s="44" t="s">
+        <v>204</v>
+      </c>
       <c r="G27" s="44"/>
-      <c r="H27" s="44"/>
-      <c r="I27" s="71"/>
+      <c r="H27" s="44" t="s">
+        <v>205</v>
+      </c>
+      <c r="I27" s="71" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="44"/>
@@ -35407,42 +35463,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -35456,18 +35512,18 @@
         <v>93</v>
       </c>
       <c r="D4" s="33" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="F4" s="34" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="24" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="B5" s="73" t="n">
         <v>0.25</v>
@@ -35479,15 +35535,15 @@
         <v>5</v>
       </c>
       <c r="E5" s="24" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="F5" s="24" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B6" s="73" t="n">
         <v>0.25</v>
@@ -35499,15 +35555,15 @@
         <v>2</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B7" s="73" t="n">
         <v>0.1</v>
@@ -35519,15 +35575,15 @@
         <v>10</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="24" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B8" s="73" t="n">
         <v>0.01</v>
@@ -35539,15 +35595,15 @@
         <v>100</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="32" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B10" s="33" t="s">
         <v>81</v>
@@ -35556,7 +35612,7 @@
         <v>83</v>
       </c>
       <c r="D10" s="33" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="E10" s="33" t="s">
         <v>102</v>
@@ -35567,83 +35623,83 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="74" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="B11" s="74" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="C11" s="74" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D11" s="74" t="s">
         <v>146</v>
       </c>
       <c r="E11" s="74" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="F11" s="74" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="74" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="B12" s="74" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="C12" s="74" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="D12" s="74" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="E12" s="74" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="F12" s="74" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="74" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="B13" s="74"/>
       <c r="C13" s="74" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="D13" s="74"/>
       <c r="E13" s="74" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="F13" s="74"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="74" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="B14" s="74"/>
       <c r="C14" s="74" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="D14" s="74"/>
       <c r="E14" s="74" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="F14" s="74"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="74" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="B15" s="74"/>
       <c r="C15" s="74" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="D15" s="74"/>
       <c r="E15" s="74" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="F15" s="74"/>
     </row>
@@ -35682,106 +35738,106 @@
   <sheetData>
     <row r="1" customFormat="false" ht="32" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="28" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="32" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="B5" s="33" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="C5" s="33" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="D5" s="33" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="E5" s="33" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="G5" s="33" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="H5" s="34" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35789,25 +35845,25 @@
         <v>1</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="C6" s="24" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D6" s="24" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="E6" s="24" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="F6" s="24" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="G6" s="24" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="H6" s="24" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35815,25 +35871,25 @@
         <v>2</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="C7" s="24" t="s">
         <v>133</v>
       </c>
       <c r="D7" s="24" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="F7" s="24" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="G7" s="24" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="H7" s="24" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35841,25 +35897,25 @@
         <v>3</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="D8" s="24" t="s">
         <v>47</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="G8" s="24" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="H8" s="24" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35867,25 +35923,25 @@
         <v>4</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="C9" s="24" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D9" s="24" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="G9" s="24" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="H9" s="24" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -35893,65 +35949,65 @@
         <v>5</v>
       </c>
       <c r="B10" s="24" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="C10" s="24" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="D10" s="24" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="G10" s="24" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="H10" s="24" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="32" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="B13" s="33" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="C13" s="33" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="D13" s="33" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="E13" s="33"/>
       <c r="F13" s="33"/>
@@ -35960,16 +36016,16 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="75" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="B14" s="76" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="C14" s="76" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="D14" s="76" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="E14" s="76"/>
       <c r="F14" s="76"/>
@@ -35978,16 +36034,16 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="77" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B15" s="76" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="C15" s="76" t="s">
         <v>98</v>
       </c>
       <c r="D15" s="76" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="E15" s="76"/>
       <c r="F15" s="76"/>
@@ -35996,16 +36052,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="78" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B16" s="76" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="C16" s="76" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="D16" s="76" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="E16" s="76"/>
       <c r="F16" s="76"/>
@@ -36014,16 +36070,16 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="79" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="B17" s="76" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="C17" s="76" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="D17" s="76" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="E17" s="76"/>
       <c r="F17" s="76"/>
@@ -36032,36 +36088,36 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="H19" s="4" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="34" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="32" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="B20" s="33" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="C20" s="33"/>
       <c r="D20" s="33"/>
@@ -36075,7 +36131,7 @@
         <v>96</v>
       </c>
       <c r="B21" s="76" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="C21" s="76"/>
       <c r="D21" s="76"/>
@@ -36089,7 +36145,7 @@
         <v>9</v>
       </c>
       <c r="B22" s="76" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="C22" s="76"/>
       <c r="D22" s="76"/>
@@ -36100,10 +36156,10 @@
     </row>
     <row r="23" customFormat="false" ht="19.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="76" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="B23" s="76" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="C23" s="76"/>
       <c r="D23" s="76"/>
@@ -36117,7 +36173,7 @@
         <v>98</v>
       </c>
       <c r="B24" s="76" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="C24" s="76"/>
       <c r="D24" s="76"/>
@@ -36131,7 +36187,7 @@
         <v>109</v>
       </c>
       <c r="B25" s="76" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="C25" s="76"/>
       <c r="D25" s="76"/>
@@ -36142,80 +36198,80 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="E27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="F27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="H27" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="F28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="H28" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="B29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="C29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="D29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="E29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="F29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="G29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="H29" s="30" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
   </sheetData>

</xml_diff>